<commit_message>
Auto: medições processadas e consolidadas
</commit_message>
<xml_diff>
--- a/CONTROLES POR COMISSÃO E GESTORES ATUALIZADA.xlsx
+++ b/CONTROLES POR COMISSÃO E GESTORES ATUALIZADA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\APRENDIZADO APP\MEDICOES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB45097E-EE60-4BEB-BA05-2EFF306343C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1EB0993-77B1-4BD3-AB1C-81F7AC4B6473}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="454" xr2:uid="{B96EB9A8-6169-46F2-89FD-740783B0C7B5}"/>
   </bookViews>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="724" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="742" uniqueCount="189">
   <si>
     <t>GESTOR(A)
 ATUANTE</t>
@@ -615,6 +615,21 @@
   </si>
   <si>
     <t>ANDERSON</t>
+  </si>
+  <si>
+    <t>330001/001196/2025</t>
+  </si>
+  <si>
+    <t>330001/001238/2025</t>
+  </si>
+  <si>
+    <t>CORDEIRO</t>
+  </si>
+  <si>
+    <t>NATIVIDADE</t>
+  </si>
+  <si>
+    <t>ENEX </t>
   </si>
 </sst>
 </file>
@@ -889,7 +904,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1004,12 +1019,674 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentagem" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="84">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -1799,659 +2476,6 @@
         <horizontal style="thin">
           <color indexed="64"/>
         </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical style="thin">
-          <color indexed="64"/>
-        </vertical>
-        <horizontal style="thin">
-          <color indexed="64"/>
-        </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -3368,43 +3392,43 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{77490B51-49AC-48CE-B9D3-F5913D37C0FB}" name="Tabela2" displayName="Tabela2" ref="B60:L75" totalsRowCount="1" headerRowDxfId="55" dataDxfId="53" totalsRowDxfId="51" headerRowBorderDxfId="54" tableBorderDxfId="52" totalsRowBorderDxfId="50">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{77490B51-49AC-48CE-B9D3-F5913D37C0FB}" name="Tabela2" displayName="Tabela2" ref="B60:L77" totalsRowCount="1" headerRowDxfId="55" dataDxfId="53" totalsRowDxfId="51" headerRowBorderDxfId="54" tableBorderDxfId="52" totalsRowBorderDxfId="50">
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{C168971F-8A1F-4CE0-AB1A-A91564F865A1}" name="GESTOR(A)_x000a_ATUANTE" totalsRowLabel="Total" dataDxfId="49" totalsRowDxfId="48"/>
-    <tableColumn id="6" xr3:uid="{28D500DA-BD33-447D-801C-1EDBD59B514A}" name="GESTOR SUPLENTE" dataDxfId="47" totalsRowDxfId="46"/>
-    <tableColumn id="2" xr3:uid="{1BC929D7-C79E-4DD8-8692-AEFFFF4E2201}" name="FISCAL NOMEADO" dataDxfId="45" totalsRowDxfId="44"/>
-    <tableColumn id="4" xr3:uid="{6DB822D5-3B20-4BEB-9FA9-33D9AE724FF4}" name="MUNICIPIO" dataDxfId="43" totalsRowDxfId="42"/>
-    <tableColumn id="5" xr3:uid="{1DE280A2-C1B5-497D-B2A7-425CC71F3653}" name="EMPRESA" totalsRowFunction="count" dataDxfId="41" totalsRowDxfId="40"/>
-    <tableColumn id="10" xr3:uid="{95ED015E-6AEE-4CBF-A570-2665B6975A98}" name="%EXEC" dataDxfId="39" totalsRowDxfId="38"/>
-    <tableColumn id="11" xr3:uid="{1C47120A-915F-4E95-BA45-AF0C41018F09}" name="STATUS" dataDxfId="37" totalsRowDxfId="36"/>
-    <tableColumn id="7" xr3:uid="{0C9C4230-87B4-46C7-8DFF-3C0A2F340B11}" name="FISCAL SUPLENTE" dataDxfId="35" totalsRowDxfId="34"/>
-    <tableColumn id="8" xr3:uid="{4E783EA6-0DCE-4695-BBAF-E24638D55153}" name="ADM" dataDxfId="33" totalsRowDxfId="32"/>
-    <tableColumn id="9" xr3:uid="{CE385090-95B6-4F49-A43B-E7EB63C58B59}" name="ADM SUPLENTE" dataDxfId="31" totalsRowDxfId="30">
+    <tableColumn id="1" xr3:uid="{C168971F-8A1F-4CE0-AB1A-A91564F865A1}" name="GESTOR(A)_x000a_ATUANTE" totalsRowLabel="Total" dataDxfId="21" totalsRowDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{28D500DA-BD33-447D-801C-1EDBD59B514A}" name="GESTOR SUPLENTE" dataDxfId="20" totalsRowDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{1BC929D7-C79E-4DD8-8692-AEFFFF4E2201}" name="FISCAL NOMEADO" dataDxfId="19" totalsRowDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{6DB822D5-3B20-4BEB-9FA9-33D9AE724FF4}" name="MUNICIPIO" dataDxfId="18" totalsRowDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{1DE280A2-C1B5-497D-B2A7-425CC71F3653}" name="EMPRESA" totalsRowFunction="count" dataDxfId="17" totalsRowDxfId="6"/>
+    <tableColumn id="10" xr3:uid="{95ED015E-6AEE-4CBF-A570-2665B6975A98}" name="%EXEC" dataDxfId="16" totalsRowDxfId="5"/>
+    <tableColumn id="11" xr3:uid="{1C47120A-915F-4E95-BA45-AF0C41018F09}" name="STATUS" dataDxfId="15" totalsRowDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{0C9C4230-87B4-46C7-8DFF-3C0A2F340B11}" name="FISCAL SUPLENTE" dataDxfId="14" totalsRowDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{4E783EA6-0DCE-4695-BBAF-E24638D55153}" name="ADM" dataDxfId="13" totalsRowDxfId="2"/>
+    <tableColumn id="9" xr3:uid="{CE385090-95B6-4F49-A43B-E7EB63C58B59}" name="ADM SUPLENTE" dataDxfId="12" totalsRowDxfId="1">
       <calculatedColumnFormula>UPPER("Rejane Vasconcelos Cristino")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{F5130F37-DBCF-45A6-A6F2-A0D5D93F0713}" name="REGIAO" dataDxfId="29" totalsRowDxfId="28"/>
+    <tableColumn id="3" xr3:uid="{F5130F37-DBCF-45A6-A6F2-A0D5D93F0713}" name="REGIAO" dataDxfId="11" totalsRowDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E49DCA8C-BF3E-4A50-9685-635EA2C8AC88}" name="Tabela3" displayName="Tabela3" ref="B38:L55" totalsRowCount="1" headerRowDxfId="27" dataDxfId="25" totalsRowDxfId="23" headerRowBorderDxfId="26" tableBorderDxfId="24" totalsRowBorderDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E49DCA8C-BF3E-4A50-9685-635EA2C8AC88}" name="Tabela3" displayName="Tabela3" ref="B38:L55" totalsRowCount="1" headerRowDxfId="49" dataDxfId="47" totalsRowDxfId="45" headerRowBorderDxfId="48" tableBorderDxfId="46" totalsRowBorderDxfId="44">
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B39:F54">
     <sortCondition ref="B38:B54"/>
   </sortState>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{7C167C76-67AF-4A26-8B9A-BCE2A4995E2A}" name="GESTOR(A)_x000a_ATUANTE" totalsRowLabel="Total" dataDxfId="21" totalsRowDxfId="20"/>
-    <tableColumn id="9" xr3:uid="{884CD221-7FDF-449F-BDDC-36A59A961922}" name="GESTOR SUPLENTE" dataDxfId="19" totalsRowDxfId="18"/>
-    <tableColumn id="2" xr3:uid="{4BAEAB60-D8F3-4A1C-A2A7-1AF80D70ECFB}" name="FISCAL NOMEADO" dataDxfId="17" totalsRowDxfId="16"/>
-    <tableColumn id="4" xr3:uid="{92B91F80-B146-424A-9B8F-B3A204D6D240}" name="MUNICIPIO" dataDxfId="15" totalsRowDxfId="14"/>
-    <tableColumn id="5" xr3:uid="{536E627B-103D-43E3-ADF4-5534C1B8AC84}" name="EMPRESA" totalsRowFunction="count" dataDxfId="13" totalsRowDxfId="12"/>
-    <tableColumn id="10" xr3:uid="{6244ECFF-D04A-4C9E-9BB6-3E00642A9BA0}" name="%EXEC" dataDxfId="11" totalsRowDxfId="10"/>
-    <tableColumn id="11" xr3:uid="{E519A9AE-567A-406C-B69A-B1B53C257A70}" name="STATUS" dataDxfId="9" totalsRowDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{682B89AE-0AB9-4B7F-8C3B-66D341320532}" name="FISCAL SUPLENTE" dataDxfId="7" totalsRowDxfId="6"/>
-    <tableColumn id="7" xr3:uid="{B76C21C5-382B-4784-B00B-25BF832EBF82}" name="ADM" dataDxfId="5" totalsRowDxfId="4"/>
-    <tableColumn id="8" xr3:uid="{E184221B-D39C-481A-9EF0-7BBC0BDCFFB3}" name="ADM SUPLENTE" dataDxfId="3" totalsRowDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{FC656C22-8A18-474F-B0C5-65DF236ED849}" name="REGIAO" dataDxfId="1" totalsRowDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{7C167C76-67AF-4A26-8B9A-BCE2A4995E2A}" name="GESTOR(A)_x000a_ATUANTE" totalsRowLabel="Total" dataDxfId="43" totalsRowDxfId="42"/>
+    <tableColumn id="9" xr3:uid="{884CD221-7FDF-449F-BDDC-36A59A961922}" name="GESTOR SUPLENTE" dataDxfId="41" totalsRowDxfId="40"/>
+    <tableColumn id="2" xr3:uid="{4BAEAB60-D8F3-4A1C-A2A7-1AF80D70ECFB}" name="FISCAL NOMEADO" dataDxfId="39" totalsRowDxfId="38"/>
+    <tableColumn id="4" xr3:uid="{92B91F80-B146-424A-9B8F-B3A204D6D240}" name="MUNICIPIO" dataDxfId="37" totalsRowDxfId="36"/>
+    <tableColumn id="5" xr3:uid="{536E627B-103D-43E3-ADF4-5534C1B8AC84}" name="EMPRESA" totalsRowFunction="count" dataDxfId="35" totalsRowDxfId="34"/>
+    <tableColumn id="10" xr3:uid="{6244ECFF-D04A-4C9E-9BB6-3E00642A9BA0}" name="%EXEC" dataDxfId="33" totalsRowDxfId="32"/>
+    <tableColumn id="11" xr3:uid="{E519A9AE-567A-406C-B69A-B1B53C257A70}" name="STATUS" dataDxfId="31" totalsRowDxfId="30"/>
+    <tableColumn id="6" xr3:uid="{682B89AE-0AB9-4B7F-8C3B-66D341320532}" name="FISCAL SUPLENTE" dataDxfId="29" totalsRowDxfId="28"/>
+    <tableColumn id="7" xr3:uid="{B76C21C5-382B-4784-B00B-25BF832EBF82}" name="ADM" dataDxfId="27" totalsRowDxfId="26"/>
+    <tableColumn id="8" xr3:uid="{E184221B-D39C-481A-9EF0-7BBC0BDCFFB3}" name="ADM SUPLENTE" dataDxfId="25" totalsRowDxfId="24"/>
+    <tableColumn id="3" xr3:uid="{FC656C22-8A18-474F-B0C5-65DF236ED849}" name="REGIAO" dataDxfId="23" totalsRowDxfId="22"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3728,7 +3752,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F61397C-D407-419C-9BDA-C160B3F745EF}">
   <sheetPr codeName="Planilha1"/>
-  <dimension ref="A1:P102"/>
+  <dimension ref="A1:P104"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.42578125" style="4" bestFit="1" customWidth="1"/>
@@ -5673,7 +5697,7 @@
 ATUANTE],N53)+COUNTIF(Tabela2[GESTOR(A)
 ATUANTE],N53)+COUNTIF(Tabela3[GESTOR(A)
 ATUANTE],N53)</f>
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="54" spans="1:16" x14ac:dyDescent="0.25">
@@ -5840,7 +5864,7 @@
         <v>183</v>
       </c>
       <c r="O60" s="36" cm="1">
-        <f t="array" ref="O60">SUMPRODUCT(IF(ISERROR(FIND(N60, $D$2:$D$74)), 0, 1))</f>
+        <f t="array" ref="O60">SUMPRODUCT(IF(ISERROR(FIND(N60, $D$2:$D$76)), 0, 1))</f>
         <v>18</v>
       </c>
       <c r="P60" s="31"/>
@@ -5886,8 +5910,8 @@
         <v>159</v>
       </c>
       <c r="O61" s="36" cm="1">
-        <f t="array" ref="O61">SUMPRODUCT(IF(ISERROR(FIND(N61, $D$2:$D$74)), 0, 1))</f>
-        <v>11</v>
+        <f t="array" ref="O61">SUMPRODUCT(IF(ISERROR(FIND(N61, $D$2:$D$76)), 0, 1))</f>
+        <v>13</v>
       </c>
       <c r="P61" s="31"/>
     </row>
@@ -5932,7 +5956,7 @@
         <v>142</v>
       </c>
       <c r="O62" s="36" cm="1">
-        <f t="array" ref="O62">SUMPRODUCT(IF(ISERROR(FIND(N62, $D$2:$D$74)), 0, 1))</f>
+        <f t="array" ref="O62">SUMPRODUCT(IF(ISERROR(FIND(N62, $D$2:$D$76)), 0, 1))</f>
         <v>0</v>
       </c>
       <c r="P62" s="31"/>
@@ -5978,7 +6002,7 @@
         <v>165</v>
       </c>
       <c r="O63" s="36" cm="1">
-        <f t="array" ref="O63">SUMPRODUCT(IF(ISERROR(FIND(N63, $D$2:$D$74)), 0, 1))</f>
+        <f t="array" ref="O63">SUMPRODUCT(IF(ISERROR(FIND(N63, $D$2:$D$76)), 0, 1))</f>
         <v>16</v>
       </c>
       <c r="P63" s="31"/>
@@ -6024,7 +6048,7 @@
         <v>139</v>
       </c>
       <c r="O64" s="36" cm="1">
-        <f t="array" ref="O64">SUMPRODUCT(IF(ISERROR(FIND(N64, $D$2:$D$74)), 0, 1))</f>
+        <f t="array" ref="O64">SUMPRODUCT(IF(ISERROR(FIND(N64, $D$2:$D$76)), 0, 1))</f>
         <v>5</v>
       </c>
       <c r="P64" s="31"/>
@@ -6070,8 +6094,8 @@
         <v>138</v>
       </c>
       <c r="O65" s="36" cm="1">
-        <f t="array" ref="O65">SUMPRODUCT(IF(ISERROR(FIND(N65, $D$2:$D$74)), 0, 1))</f>
-        <v>6</v>
+        <f t="array" ref="O65">SUMPRODUCT(IF(ISERROR(FIND(N65, $D$2:$D$76)), 0, 1))</f>
+        <v>8</v>
       </c>
       <c r="P65" s="31"/>
     </row>
@@ -6116,7 +6140,7 @@
         <v>158</v>
       </c>
       <c r="O66" s="36" cm="1">
-        <f t="array" ref="O66">SUMPRODUCT(IF(ISERROR(FIND(N66, $D$2:$D$74)), 0, 1))</f>
+        <f t="array" ref="O66">SUMPRODUCT(IF(ISERROR(FIND(N66, $D$2:$D$76)), 0, 1))</f>
         <v>16</v>
       </c>
       <c r="P66" s="31"/>
@@ -6162,7 +6186,7 @@
         <v>145</v>
       </c>
       <c r="O67" s="36" cm="1">
-        <f t="array" ref="O67">SUMPRODUCT(IF(ISERROR(FIND(N67, $D$2:$D$74)), 0, 1))</f>
+        <f t="array" ref="O67">SUMPRODUCT(IF(ISERROR(FIND(N67, $D$2:$D$76)), 0, 1))</f>
         <v>17</v>
       </c>
       <c r="P67" s="31"/>
@@ -6196,7 +6220,7 @@
         <v>148</v>
       </c>
       <c r="J68" s="15" t="str">
-        <f t="shared" ref="J68:J74" si="0">UPPER("REJANE VASCONCELOS")</f>
+        <f t="shared" ref="J68:J76" si="0">UPPER("REJANE VASCONCELOS")</f>
         <v>REJANE VASCONCELOS</v>
       </c>
       <c r="K68" s="15" t="s">
@@ -6209,7 +6233,7 @@
         <v>143</v>
       </c>
       <c r="O68" s="36" cm="1">
-        <f t="array" ref="O68">SUMPRODUCT(IF(ISERROR(FIND(N68, $D$2:$D$74)), 0, 1))</f>
+        <f t="array" ref="O68">SUMPRODUCT(IF(ISERROR(FIND(N68, $D$2:$D$76)), 0, 1))</f>
         <v>1</v>
       </c>
       <c r="P68" s="31"/>
@@ -6255,7 +6279,7 @@
         <v>161</v>
       </c>
       <c r="O69" s="36" cm="1">
-        <f t="array" ref="O69">SUMPRODUCT(IF(ISERROR(FIND(N69, $D$2:$D$74)), 0, 1))</f>
+        <f t="array" ref="O69">SUMPRODUCT(IF(ISERROR(FIND(N69, $D$2:$D$76)), 0, 1))</f>
         <v>0</v>
       </c>
       <c r="P69" s="31"/>
@@ -6302,96 +6326,90 @@
         <v>144</v>
       </c>
       <c r="O70" s="36" cm="1">
-        <f t="array" ref="O70">SUMPRODUCT(IF(ISERROR(FIND(N70, $D$2:$D$74)), 0, 1))</f>
+        <f t="array" ref="O70">SUMPRODUCT(IF(ISERROR(FIND(N70, $D$2:$D$76)), 0, 1))</f>
         <v>18</v>
       </c>
       <c r="P70" s="31"/>
     </row>
     <row r="71" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A71" s="39" t="s">
-        <v>53</v>
+      <c r="A71" s="48" t="s">
+        <v>184</v>
       </c>
       <c r="B71" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C71" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="D71" s="6" t="s">
-        <v>150</v>
+      <c r="D71" s="21" t="s">
+        <v>149</v>
       </c>
       <c r="E71" s="6" t="s">
-        <v>64</v>
+        <v>186</v>
       </c>
       <c r="F71" s="21" t="s">
-        <v>133</v>
-      </c>
-      <c r="G71" s="28">
-        <v>0.87860000000000005</v>
-      </c>
-      <c r="H71" s="21" t="s">
-        <v>153</v>
-      </c>
-      <c r="I71" s="21" t="s">
-        <v>148</v>
-      </c>
-      <c r="J71" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>REJANE VASCONCELOS</v>
-      </c>
-      <c r="K71" s="6" t="s">
-        <v>132</v>
+        <v>119</v>
+      </c>
+      <c r="G71" s="54"/>
+      <c r="H71" s="55"/>
+      <c r="I71" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="J71" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="K71" s="56" t="str">
+        <f t="shared" ref="K71:K72" si="1">UPPER("Rejane Vasconcelos Cristino")</f>
+        <v>REJANE VASCONCELOS CRISTINO</v>
       </c>
       <c r="L71" s="43" t="s">
         <v>170</v>
       </c>
-      <c r="N71"/>
-      <c r="O71" s="31"/>
+      <c r="N71" s="52"/>
+      <c r="O71" s="53"/>
       <c r="P71" s="31"/>
     </row>
     <row r="72" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A72" s="40" t="s">
-        <v>120</v>
+      <c r="A72" s="48" t="s">
+        <v>185</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C72" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="D72" s="6" t="s">
-        <v>150</v>
+      <c r="D72" s="21" t="s">
+        <v>149</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>121</v>
+        <v>187</v>
       </c>
       <c r="F72" s="21" t="s">
-        <v>122</v>
-      </c>
-      <c r="G72" s="28">
-        <v>0</v>
-      </c>
-      <c r="H72" s="21" t="s">
-        <v>153</v>
-      </c>
-      <c r="I72" s="21" t="s">
-        <v>148</v>
-      </c>
-      <c r="J72" s="6" t="str">
-        <f t="shared" si="0"/>
-        <v>REJANE VASCONCELOS</v>
-      </c>
-      <c r="K72" s="6" t="s">
-        <v>132</v>
+        <v>188</v>
+      </c>
+      <c r="G72" s="54"/>
+      <c r="H72" s="55"/>
+      <c r="I72" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="J72" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="K72" s="56" t="str">
+        <f t="shared" si="1"/>
+        <v>REJANE VASCONCELOS CRISTINO</v>
       </c>
       <c r="L72" s="43" t="s">
         <v>170</v>
       </c>
-      <c r="N72"/>
+      <c r="N72" s="52"/>
+      <c r="O72" s="53"/>
+      <c r="P72" s="31"/>
     </row>
     <row r="73" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A73" s="39" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B73" s="5" t="s">
         <v>138</v>
@@ -6403,13 +6421,13 @@
         <v>150</v>
       </c>
       <c r="E73" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F73" s="21" t="s">
-        <v>66</v>
+        <v>133</v>
       </c>
       <c r="G73" s="28">
-        <v>0.97019999999999995</v>
+        <v>0.87860000000000005</v>
       </c>
       <c r="H73" s="21" t="s">
         <v>153</v>
@@ -6428,28 +6446,30 @@
         <v>170</v>
       </c>
       <c r="N73"/>
+      <c r="O73" s="31"/>
+      <c r="P73" s="31"/>
     </row>
     <row r="74" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A74" s="40" t="s">
-        <v>55</v>
-      </c>
-      <c r="B74" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="B74" s="5" t="s">
         <v>138</v>
       </c>
       <c r="C74" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="D74" s="9" t="s">
+      <c r="D74" s="6" t="s">
         <v>150</v>
       </c>
-      <c r="E74" s="9" t="s">
-        <v>67</v>
+      <c r="E74" s="6" t="s">
+        <v>121</v>
       </c>
       <c r="F74" s="21" t="s">
-        <v>68</v>
+        <v>122</v>
       </c>
       <c r="G74" s="28">
-        <v>0.31530000000000002</v>
+        <v>0</v>
       </c>
       <c r="H74" s="21" t="s">
         <v>153</v>
@@ -6470,70 +6490,140 @@
       <c r="N74"/>
     </row>
     <row r="75" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A75" s="23"/>
-      <c r="B75" s="8" t="s">
+      <c r="A75" s="39" t="s">
+        <v>54</v>
+      </c>
+      <c r="B75" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="C75" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="D75" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="E75" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="F75" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="G75" s="28">
+        <v>0.97019999999999995</v>
+      </c>
+      <c r="H75" s="21" t="s">
+        <v>153</v>
+      </c>
+      <c r="I75" s="21" t="s">
+        <v>148</v>
+      </c>
+      <c r="J75" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v>REJANE VASCONCELOS</v>
+      </c>
+      <c r="K75" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="L75" s="43" t="s">
+        <v>170</v>
+      </c>
+      <c r="N75"/>
+    </row>
+    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A76" s="40" t="s">
+        <v>55</v>
+      </c>
+      <c r="B76" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="C76" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="D76" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="E76" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="F76" s="21" t="s">
+        <v>68</v>
+      </c>
+      <c r="G76" s="28">
+        <v>0.31530000000000002</v>
+      </c>
+      <c r="H76" s="21" t="s">
+        <v>153</v>
+      </c>
+      <c r="I76" s="21" t="s">
+        <v>148</v>
+      </c>
+      <c r="J76" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v>REJANE VASCONCELOS</v>
+      </c>
+      <c r="K76" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="L76" s="43" t="s">
+        <v>170</v>
+      </c>
+      <c r="N76"/>
+    </row>
+    <row r="77" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A77" s="23"/>
+      <c r="B77" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="C75" s="8"/>
-      <c r="D75" s="9"/>
-      <c r="E75" s="9"/>
-      <c r="F75" s="14">
+      <c r="C77" s="8"/>
+      <c r="D77" s="9"/>
+      <c r="E77" s="9"/>
+      <c r="F77" s="14">
         <f>SUBTOTAL(103,Tabela2[EMPRESA])</f>
-        <v>14</v>
-      </c>
-      <c r="G75" s="14"/>
-      <c r="H75" s="14"/>
-      <c r="I75" s="9"/>
-      <c r="J75" s="9"/>
-      <c r="K75" s="9"/>
-      <c r="L75" s="9"/>
-      <c r="N75"/>
-    </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B76" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G77" s="14"/>
+      <c r="H77" s="14"/>
+      <c r="I77" s="9"/>
+      <c r="J77" s="9"/>
+      <c r="K77" s="9"/>
+      <c r="L77" s="9"/>
+      <c r="N77"/>
+    </row>
+    <row r="78" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B78" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="C76" s="13">
+      <c r="C78" s="13">
         <f>COUNTIF(Tabela2[GESTOR(A)
-ATUANTE],B76)</f>
-        <v>7</v>
-      </c>
-      <c r="O76" s="31"/>
-    </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B77" s="6" t="s">
+ATUANTE],B78)</f>
+        <v>9</v>
+      </c>
+      <c r="O78" s="31"/>
+    </row>
+    <row r="79" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="B79" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="C77" s="13">
+      <c r="C79" s="13">
         <f>COUNTIF(Tabela2[GESTOR(A)
-ATUANTE],B77)</f>
+ATUANTE],B79)</f>
         <v>5</v>
       </c>
-      <c r="O77" s="31"/>
-    </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="O78" s="31"/>
-    </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B79"/>
-      <c r="C79"/>
-      <c r="D79"/>
-      <c r="E79"/>
-      <c r="F79"/>
       <c r="O79" s="31"/>
     </row>
     <row r="80" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="D80" s="23"/>
-      <c r="E80"/>
-      <c r="F80"/>
       <c r="O80" s="31"/>
     </row>
     <row r="81" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B81"/>
+      <c r="C81"/>
+      <c r="D81"/>
       <c r="E81"/>
       <c r="F81"/>
       <c r="O81" s="31"/>
     </row>
     <row r="82" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="D82" s="23"/>
       <c r="E82"/>
       <c r="F82"/>
       <c r="O82" s="31"/>
@@ -6549,28 +6639,30 @@
       <c r="O84" s="31"/>
     </row>
     <row r="85" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="G85" s="4"/>
+      <c r="E85"/>
+      <c r="F85"/>
       <c r="O85" s="31"/>
     </row>
     <row r="86" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B86"/>
-      <c r="C86"/>
-      <c r="D86"/>
-      <c r="G86" s="4"/>
+      <c r="E86"/>
+      <c r="F86"/>
       <c r="O86" s="31"/>
     </row>
     <row r="87" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B87"/>
-      <c r="C87"/>
-      <c r="D87"/>
       <c r="G87" s="4"/>
       <c r="O87" s="31"/>
     </row>
     <row r="88" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B88"/>
+      <c r="C88"/>
+      <c r="D88"/>
       <c r="G88" s="4"/>
       <c r="O88" s="31"/>
     </row>
     <row r="89" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B89"/>
+      <c r="C89"/>
+      <c r="D89"/>
       <c r="G89" s="4"/>
       <c r="O89" s="31"/>
     </row>
@@ -6579,17 +6671,17 @@
       <c r="O90" s="31"/>
     </row>
     <row r="91" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="E91"/>
-      <c r="F91"/>
+      <c r="G91" s="4"/>
       <c r="O91" s="31"/>
     </row>
-    <row r="95" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="H95"/>
-      <c r="I95"/>
-    </row>
-    <row r="96" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="H96"/>
-      <c r="I96"/>
+    <row r="92" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="G92" s="4"/>
+      <c r="O92" s="31"/>
+    </row>
+    <row r="93" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="E93"/>
+      <c r="F93"/>
+      <c r="O93" s="31"/>
     </row>
     <row r="97" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H97"/>
@@ -6614,6 +6706,14 @@
     <row r="102" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H102"/>
       <c r="I102"/>
+    </row>
+    <row r="103" spans="8:9" x14ac:dyDescent="0.25">
+      <c r="H103"/>
+      <c r="I103"/>
+    </row>
+    <row r="104" spans="8:9" x14ac:dyDescent="0.25">
+      <c r="H104"/>
+      <c r="I104"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:A33" xr:uid="{4F61397C-D407-419C-9BDA-C160B3F745EF}"/>
@@ -6632,7 +6732,7 @@
     <oddFooter>Página &amp;P de &amp;N</oddFooter>
   </headerFooter>
   <ignoredErrors>
-    <ignoredError sqref="K61:K69 K71:K74" calculatedColumn="1"/>
+    <ignoredError sqref="K61:K70 K73:K76" calculatedColumn="1"/>
   </ignoredErrors>
   <tableParts count="3">
     <tablePart r:id="rId2"/>

</xml_diff>